<commit_message>
Add a November test section built from the Biology checklist
The school's Year 9-10 checklist (127 statements) decides exactly which
Biology cards are on the test: everything except stem cells, the nervous
system, eye and plant responses, inheritance, and selective breeding, GM
and cloning. Those cards are tagged and gathered into a 'November test -
Biology' deck in Flashcards, moving only cards that change, and go back
to the Biology deck after the test.

The study plan now has the checklist to rate statement by statement.
Topic priority combines those ratings with flashcard confidence, and the
day-by-day sprint names the topic for each session in priority order,
with question practice on the previous day's topic. The workbook tracker
matches the checklist.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MRVKNvUVmqxD1S6v3u9v6z
</commit_message>
<xml_diff>
--- a/study-plan/GCSE_Study_Plan.xlsx
+++ b/study-plan/GCSE_Study_Plan.xlsx
@@ -206,7 +206,7 @@
     <t xml:space="preserve">Yes</t>
   </si>
   <si>
-    <t xml:space="preserve">2a–b Cells and organisation</t>
+    <t xml:space="preserve">2a–b Cells and organisation (not stem cells)</t>
   </si>
   <si>
     <t xml:space="preserve">2c Biological molecules (incl. enzymes, food tests)</t>
@@ -233,28 +233,28 @@
     <t xml:space="preserve">2i Excretion</t>
   </si>
   <si>
+    <t xml:space="preserve">2j Coordination and response (not nervous system, eye, plant responses)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3a Reproduction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3b Inheritance – NOT on the test</t>
+  </si>
+  <si>
     <t xml:space="preserve">No</t>
   </si>
   <si>
-    <t xml:space="preserve">2j Coordination and response</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3a Reproduction</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3b Inheritance</t>
-  </si>
-  <si>
     <t xml:space="preserve">4 Ecology and environment</t>
   </si>
   <si>
-    <t xml:space="preserve">5 Use of biological resources</t>
+    <t xml:space="preserve">5 Use of biological resources (not selective breeding, GM, cloning)</t>
   </si>
   <si>
     <t xml:space="preserve">Topics on the test</t>
   </si>
   <si>
-    <t xml:space="preserve">Which Year 9–10 topics are tested is a guess (topics 1–2h) – set "On the test?" to match what your teacher said. Orange rows = revise first. In the app, study just these topics with Flashcards → Browse/Custom study (search e.g. deck:"Biology::2h*"), and blurt each one in Tools → Blurting.</t>
+    <t xml:space="preserve">From your school checklist: all of Biology except stem cells, the nervous system / eye / plant responses, inheritance, and selective breeding / GM / cloning. Orange rows = revise first. In the app, the "November test – Biology" flashcard deck has exactly these cards, and Tools → Study plan has the full checklist to rate. In the app, study just these topics with Flashcards → Browse/Custom study (search e.g. deck:"Biology::2h*"), and blurt each one in Tools → Blurting.</t>
   </si>
   <si>
     <t xml:space="preserve">English Language skills tracker (assumed Edexcel IGCSE English Language A, 4EA1)</t>
@@ -440,7 +440,7 @@
     <t xml:space="preserve">0 November tests</t>
   </si>
   <si>
-    <t xml:space="preserve">Biology (Year 9–10 topics) and English Language tests in early November – see the November tests sheet.</t>
+    <t xml:space="preserve">Biology (everything on the Year 9–10 checklist) and English Language tests in early November – see the November tests sheet.</t>
   </si>
   <si>
     <t xml:space="preserve">All due cards daily (all subjects); Biology cards first</t>
@@ -2168,7 +2168,7 @@
       <c r="F11" s="16"/>
       <c r="G11" s="16"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
         <v>52</v>
       </c>
@@ -2317,32 +2317,32 @@
         <v>60</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="C20" s="14" t="n">
         <v>3</v>
       </c>
       <c r="D20" s="15" t="n">
         <f aca="false">IF(B20="Yes",6-C20,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E20" s="16"/>
       <c r="F20" s="16"/>
       <c r="G20" s="16"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="C21" s="14" t="n">
         <v>3</v>
       </c>
       <c r="D21" s="15" t="n">
         <f aca="false">IF(B21="Yes",6-C21,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E21" s="16"/>
       <c r="F21" s="16"/>
@@ -2350,17 +2350,17 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="C22" s="14" t="n">
         <v>3</v>
       </c>
       <c r="D22" s="15" t="n">
         <f aca="false">IF(B22="Yes",6-C22,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E22" s="16"/>
       <c r="F22" s="16"/>
@@ -2368,10 +2368,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="B23" s="14" t="s">
         <v>64</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>61</v>
       </c>
       <c r="C23" s="14" t="n">
         <v>3</v>
@@ -2389,32 +2389,32 @@
         <v>65</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="C24" s="14" t="n">
         <v>3</v>
       </c>
       <c r="D24" s="15" t="n">
         <f aca="false">IF(B24="Yes",6-C24,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E24" s="16"/>
       <c r="F24" s="16"/>
       <c r="G24" s="16"/>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
         <v>66</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="C25" s="14" t="n">
         <v>3</v>
       </c>
       <c r="D25" s="15" t="n">
         <f aca="false">IF(B25="Yes",6-C25,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E25" s="16"/>
       <c r="F25" s="16"/>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="B26" s="6" t="n">
         <f aca="false">COUNTIF(B11:B25,"Yes")</f>
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="F41" s="13"/>
       <c r="G41" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2656,7 +2656,7 @@
       </c>
       <c r="F42" s="13"/>
       <c r="G42" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2676,7 +2676,7 @@
       <c r="E43" s="13"/>
       <c r="F43" s="13"/>
       <c r="G43" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2700,7 +2700,7 @@
         <v>104</v>
       </c>
       <c r="G44" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2724,7 +2724,7 @@
         <v>107</v>
       </c>
       <c r="G45" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2746,7 +2746,7 @@
       </c>
       <c r="F46" s="13"/>
       <c r="G46" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="F47" s="13"/>
       <c r="G47" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2790,7 +2790,7 @@
       </c>
       <c r="F48" s="13"/>
       <c r="G48" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="F49" s="13"/>
       <c r="G49" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2832,7 +2832,7 @@
       <c r="E50" s="13"/>
       <c r="F50" s="13"/>
       <c r="G50" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2856,7 +2856,7 @@
         <v>108</v>
       </c>
       <c r="G51" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2880,7 +2880,7 @@
         <v>109</v>
       </c>
       <c r="G52" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2902,7 +2902,7 @@
       </c>
       <c r="F53" s="13"/>
       <c r="G53" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2924,7 +2924,7 @@
       </c>
       <c r="F54" s="13"/>
       <c r="G54" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2946,7 +2946,7 @@
       </c>
       <c r="F55" s="13"/>
       <c r="G55" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2968,7 +2968,7 @@
       </c>
       <c r="F56" s="13"/>
       <c r="G56" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2988,7 +2988,7 @@
       <c r="E57" s="13"/>
       <c r="F57" s="13"/>
       <c r="G57" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3012,7 +3012,7 @@
         <v>108</v>
       </c>
       <c r="G58" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="F59" s="13"/>
       <c r="G59" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3054,7 +3054,7 @@
       <c r="E60" s="13"/>
       <c r="F60" s="13"/>
       <c r="G60" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3074,7 +3074,7 @@
       <c r="E61" s="13"/>
       <c r="F61" s="13"/>
       <c r="G61" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3184,7 +3184,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="22" t="s">
         <v>129</v>
       </c>
@@ -5434,7 +5434,7 @@
         <v>2</v>
       </c>
       <c r="I5" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J5" s="16"/>
     </row>
@@ -5466,7 +5466,7 @@
         <v>2</v>
       </c>
       <c r="I6" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J6" s="16"/>
     </row>
@@ -5498,7 +5498,7 @@
         <v>2</v>
       </c>
       <c r="I7" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J7" s="16"/>
     </row>
@@ -5530,7 +5530,7 @@
         <v>1</v>
       </c>
       <c r="I8" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J8" s="16"/>
     </row>
@@ -5562,7 +5562,7 @@
         <v>1</v>
       </c>
       <c r="I9" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J9" s="16"/>
     </row>
@@ -5594,7 +5594,7 @@
         <v>1</v>
       </c>
       <c r="I10" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J10" s="16"/>
     </row>
@@ -5626,7 +5626,7 @@
         <v>1</v>
       </c>
       <c r="I11" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J11" s="16"/>
     </row>
@@ -5658,7 +5658,7 @@
         <v>1</v>
       </c>
       <c r="I12" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J12" s="16"/>
     </row>
@@ -5690,7 +5690,7 @@
         <v>1</v>
       </c>
       <c r="I13" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J13" s="16"/>
     </row>
@@ -5722,7 +5722,7 @@
         <v>5</v>
       </c>
       <c r="I14" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J14" s="16"/>
     </row>
@@ -5754,7 +5754,7 @@
         <v>5</v>
       </c>
       <c r="I15" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J15" s="16"/>
     </row>
@@ -5786,7 +5786,7 @@
         <v>5</v>
       </c>
       <c r="I16" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J16" s="16"/>
     </row>
@@ -5818,7 +5818,7 @@
         <v>5</v>
       </c>
       <c r="I17" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J17" s="16"/>
     </row>
@@ -5850,7 +5850,7 @@
         <v>5</v>
       </c>
       <c r="I18" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J18" s="16"/>
     </row>
@@ -5882,7 +5882,7 @@
         <v>6</v>
       </c>
       <c r="I19" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J19" s="16"/>
     </row>
@@ -5914,7 +5914,7 @@
         <v>6</v>
       </c>
       <c r="I20" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J20" s="16"/>
     </row>
@@ -5946,7 +5946,7 @@
         <v>6</v>
       </c>
       <c r="I21" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J21" s="16"/>
     </row>
@@ -5978,7 +5978,7 @@
         <v>6</v>
       </c>
       <c r="I22" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J22" s="16"/>
     </row>
@@ -6010,7 +6010,7 @@
         <v>6</v>
       </c>
       <c r="I23" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J23" s="16"/>
     </row>
@@ -6042,7 +6042,7 @@
         <v>6</v>
       </c>
       <c r="I24" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J24" s="16"/>
     </row>
@@ -6074,7 +6074,7 @@
         <v>6</v>
       </c>
       <c r="I25" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J25" s="16"/>
     </row>
@@ -6106,7 +6106,7 @@
         <v>6</v>
       </c>
       <c r="I26" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J26" s="16"/>
     </row>
@@ -6138,7 +6138,7 @@
         <v>6</v>
       </c>
       <c r="I27" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J27" s="16"/>
     </row>
@@ -6170,7 +6170,7 @@
         <v>6</v>
       </c>
       <c r="I28" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J28" s="16"/>
     </row>
@@ -6202,7 +6202,7 @@
         <v>10</v>
       </c>
       <c r="I29" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J29" s="16"/>
     </row>
@@ -6234,7 +6234,7 @@
         <v>10</v>
       </c>
       <c r="I30" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J30" s="16"/>
     </row>
@@ -6266,7 +6266,7 @@
         <v>10</v>
       </c>
       <c r="I31" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J31" s="16"/>
     </row>
@@ -6298,7 +6298,7 @@
         <v>6</v>
       </c>
       <c r="I32" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J32" s="16"/>
     </row>
@@ -6330,7 +6330,7 @@
         <v>6</v>
       </c>
       <c r="I33" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J33" s="16"/>
     </row>
@@ -6362,7 +6362,7 @@
         <v>6</v>
       </c>
       <c r="I34" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J34" s="16"/>
     </row>
@@ -6394,7 +6394,7 @@
         <v>6</v>
       </c>
       <c r="I35" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J35" s="16"/>
     </row>
@@ -6426,7 +6426,7 @@
         <v>6</v>
       </c>
       <c r="I36" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J36" s="16"/>
     </row>
@@ -6458,7 +6458,7 @@
         <v>6</v>
       </c>
       <c r="I37" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J37" s="16"/>
     </row>
@@ -6490,7 +6490,7 @@
         <v>6</v>
       </c>
       <c r="I38" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J38" s="16"/>
     </row>
@@ -6522,7 +6522,7 @@
         <v>6</v>
       </c>
       <c r="I39" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J39" s="16"/>
     </row>
@@ -6554,7 +6554,7 @@
         <v>6</v>
       </c>
       <c r="I40" s="21" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J40" s="16"/>
     </row>

</xml_diff>